<commit_message>
Add more entries for missing quest and gossip audio, and some corrections/modifications
</commit_message>
<xml_diff>
--- a/corrections/corrections.xlsx
+++ b/corrections/corrections.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\Desktop\wow_vo_webui\corrections\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05146EB0-B3AE-4516-920B-AA2ABDDDF7B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{907DA846-7FE7-4A0A-A15C-7B2FD7261A56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="quest" sheetId="2" r:id="rId1"/>
@@ -20,17 +20,26 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">npc!$A$1:$H$778</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">quest!$A$1:$F$1343</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1294" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1308" uniqueCount="365">
   <si>
     <t>source</t>
   </si>
@@ -1460,6 +1469,20 @@
   </si>
   <si>
     <t>A rune circle? dragonkin? The Defias have allied themselves with HER? The traitor?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">It is no longer my purpose to hunt, but to teach the hunter. That is what fate has handed to me. Craft with me a hunter's charm, a collection of trophies from fallen prey that will remind you of your past trials and triumphs. In the end I will keep the charm, but reward you with something else. </t>
+  </si>
+  <si>
+    <t>You place the gem inside the essence font.
+Thank you mortal, you have - no; this, this cannot be! No!  The corruption of this accursed god even taints the sanctity of a Green Dragonflight essence font!  No please, I feel my essence ripping from me!  THE PAIN!  I feel the grip of an eternal nightmare taking hold on me.
+Mortal, I implore you!  Find one of the Green Dragonflight to stop this; help me; I am chained in darkness; forever in agony; please do not torture."</t>
+  </si>
+  <si>
+    <t>You have learned the old ways, adventurer, and for that, I offer you a gift from my days as a hunter.</t>
+  </si>
+  <si>
+    <t>The cry for vengeance must be heard, adventurer. Commander Plague-fist and a company of death knights are on their way to raze the Chapel of the Crimson Flame. If there are any death knights imprisoned at the chapel, Plague-fist will get them out. You can still catch up to them if you hurry; The chapel is due west of here.</t>
   </si>
 </sst>
 </file>
@@ -1495,8 +1518,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1858,7 +1882,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56545B79-22C0-4057-A076-1E697524330B}">
-  <dimension ref="A1:F1360"/>
+  <dimension ref="A1:F1368"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -13648,6 +13672,94 @@
       </c>
       <c r="F1360" t="s">
         <v>226</v>
+      </c>
+    </row>
+    <row r="1361" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1361" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1361">
+        <v>5204</v>
+      </c>
+      <c r="F1361" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1362" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1362" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1362">
+        <v>5385</v>
+      </c>
+      <c r="F1362" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1363" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1363" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1363">
+        <v>8233</v>
+      </c>
+      <c r="E1363">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1364" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1364" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1364">
+        <v>8417</v>
+      </c>
+      <c r="E1364">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1365" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1365" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1365">
+        <v>8151</v>
+      </c>
+      <c r="D1365" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="1366" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1366" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1366">
+        <v>3373</v>
+      </c>
+      <c r="D1366" s="1" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="1367" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1367" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1367">
+        <v>8232</v>
+      </c>
+      <c r="D1367" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="1368" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1368" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1368">
+        <v>12738</v>
+      </c>
+      <c r="D1368" t="s">
+        <v>364</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add more entries based on gameplay feedback
</commit_message>
<xml_diff>
--- a/corrections/corrections.xlsx
+++ b/corrections/corrections.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\Desktop\wow_vo_webui\corrections\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{907DA846-7FE7-4A0A-A15C-7B2FD7261A56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{131987BF-47AE-4204-B8A4-B4A9FF3BF2FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="quest" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1308" uniqueCount="365">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1313" uniqueCount="365">
   <si>
     <t>source</t>
   </si>
@@ -13778,7 +13778,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D60A7C4-82C4-4AAF-A00A-127D625F91A3}">
-  <dimension ref="A1:H876"/>
+  <dimension ref="A1:H881"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -18605,6 +18605,12 @@
       <c r="A572">
         <v>28615</v>
       </c>
+      <c r="C572">
+        <v>42</v>
+      </c>
+      <c r="D572">
+        <v>0</v>
+      </c>
       <c r="E572" t="s">
         <v>29</v>
       </c>
@@ -18613,6 +18619,12 @@
       <c r="A573">
         <v>29480</v>
       </c>
+      <c r="C573">
+        <v>42</v>
+      </c>
+      <c r="D573">
+        <v>0</v>
+      </c>
       <c r="E573" t="s">
         <v>29</v>
       </c>
@@ -18621,6 +18633,12 @@
       <c r="A574">
         <v>31078</v>
       </c>
+      <c r="C574">
+        <v>42</v>
+      </c>
+      <c r="D574">
+        <v>0</v>
+      </c>
       <c r="E574" t="s">
         <v>29</v>
       </c>
@@ -19118,6 +19136,12 @@
       <c r="B635">
         <v>0</v>
       </c>
+      <c r="C635">
+        <v>9</v>
+      </c>
+      <c r="D635">
+        <v>0</v>
+      </c>
       <c r="E635" t="s">
         <v>17</v>
       </c>
@@ -20788,6 +20812,12 @@
       <c r="A843">
         <v>10583</v>
       </c>
+      <c r="C843">
+        <v>9</v>
+      </c>
+      <c r="D843">
+        <v>0</v>
+      </c>
       <c r="E843" t="s">
         <v>17</v>
       </c>
@@ -21057,6 +21087,79 @@
       </c>
       <c r="E876" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="877" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A877">
+        <v>18938</v>
+      </c>
+      <c r="C877">
+        <v>9</v>
+      </c>
+      <c r="D877">
+        <v>0</v>
+      </c>
+      <c r="E877" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="878" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A878">
+        <v>19583</v>
+      </c>
+      <c r="C878">
+        <v>9</v>
+      </c>
+      <c r="D878">
+        <v>0</v>
+      </c>
+      <c r="E878" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="879" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A879">
+        <v>20515</v>
+      </c>
+      <c r="C879">
+        <v>9</v>
+      </c>
+      <c r="D879">
+        <v>0</v>
+      </c>
+      <c r="E879" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="880" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A880">
+        <v>23612</v>
+      </c>
+      <c r="C880">
+        <v>9</v>
+      </c>
+      <c r="D880">
+        <v>0</v>
+      </c>
+      <c r="E880" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="881" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A881">
+        <v>24366</v>
+      </c>
+      <c r="B881">
+        <v>1</v>
+      </c>
+      <c r="C881">
+        <v>9</v>
+      </c>
+      <c r="D881">
+        <v>0</v>
+      </c>
+      <c r="E881" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>